<commit_message>
updates to 4 scripts + misc. clean ups
Normunit updates (placeholder value for Commercial Cap-tons)
Helper function to extract starting day of week (for Source Year) for simulation for CEDARS format
Rearranged CEDARS code snippet position for better traceability
Updated gitignore for generated outputs
</commit_message>
<xml_diff>
--- a/scripts/data transformation/Normunits.xlsx
+++ b/scripts/data transformation/Normunits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YLIAN\Documents\DEER_github_2026\DEER-Prototypes-EnergyPlus\scripts\data transformation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0476B37-B39C-491B-A492-96260E112D89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE893D6-139A-4B4D-8A6A-C47785252B00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{527A75FC-5BC9-4372-9120-09678A46B600}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{527A75FC-5BC9-4372-9120-09678A46B600}"/>
   </bookViews>
   <sheets>
     <sheet name="DMo" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Update Normunit logic with validation + lookup
</commit_message>
<xml_diff>
--- a/scripts/data transformation/Normunits.xlsx
+++ b/scripts/data transformation/Normunits.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YLIAN\Documents\DEER_github_2026\DEER-Prototypes-EnergyPlus\scripts\data transformation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YLIAN\Documents\DEER_github_apr26\DEER-Prototypes-EnergyPlus\scripts\data transformation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C39AEBF-6923-416F-AEF8-65544804267E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FE080E6-8019-465C-8D28-A823225A6BBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{527A75FC-5BC9-4372-9120-09678A46B600}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{527A75FC-5BC9-4372-9120-09678A46B600}"/>
   </bookViews>
   <sheets>
     <sheet name="DMo" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="83">
   <si>
     <t>Normunit</t>
   </si>
@@ -280,9 +280,6 @@
     <t>added 7/18/2024 to accommodate Normunit = Each</t>
   </si>
   <si>
-    <t>Cap-Ton</t>
-  </si>
-  <si>
     <t>3/3/2026 Placeholder value here to test Com.py script for consistency. Correct capacity from each building type model needs to be extracted and placed here.</t>
   </si>
   <si>
@@ -320,6 +317,15 @@
   </si>
   <si>
     <t>meas_area converted to ft2</t>
+  </si>
+  <si>
+    <t>Fallback normunit if all else not matching, please make sure it matches</t>
+  </si>
+  <si>
+    <t>Windows</t>
+  </si>
+  <si>
+    <t>6/11/26: Placeholder value, please update for windows</t>
   </si>
 </sst>
 </file>
@@ -329,7 +335,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -342,12 +348,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -710,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2593147D-FBCE-4A43-B94C-18CB04EC4F0B}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
@@ -775,33 +775,50 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
       <c r="C5">
+        <v>2000</v>
+      </c>
+      <c r="D5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6">
         <f>400*2</f>
         <v>800</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" t="s">
         <v>3</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>3.5</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D7" t="s">
         <v>56</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E7" t="s">
         <v>54</v>
       </c>
     </row>
@@ -813,7 +830,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C9AEBA2-4873-4E93-88D1-6559970F8CAA}">
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
@@ -881,30 +898,30 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C5">
-        <v>19.45</v>
+        <v>5000</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" t="s">
-        <v>23</v>
+        <v>81</v>
+      </c>
+      <c r="F5" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6">
-        <v>22.32</v>
+        <v>19.45</v>
       </c>
       <c r="D6" t="s">
         <v>24</v>
@@ -915,13 +932,13 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C7">
-        <v>24.49</v>
+        <v>22.32</v>
       </c>
       <c r="D7" t="s">
         <v>24</v>
@@ -932,13 +949,13 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C8">
-        <v>23.49</v>
+        <v>24.49</v>
       </c>
       <c r="D8" t="s">
         <v>24</v>
@@ -949,13 +966,13 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9">
-        <v>23.88</v>
+        <v>23.49</v>
       </c>
       <c r="D9" t="s">
         <v>24</v>
@@ -966,13 +983,13 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10">
-        <v>23.79</v>
+        <v>23.88</v>
       </c>
       <c r="D10" t="s">
         <v>24</v>
@@ -983,13 +1000,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C11">
-        <v>22.48</v>
+        <v>23.79</v>
       </c>
       <c r="D11" t="s">
         <v>24</v>
@@ -1000,13 +1017,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C12">
-        <v>27.59</v>
+        <v>22.48</v>
       </c>
       <c r="D12" t="s">
         <v>24</v>
@@ -1017,13 +1034,13 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13">
-        <v>35.33</v>
+        <v>27.59</v>
       </c>
       <c r="D13" t="s">
         <v>24</v>
@@ -1034,13 +1051,13 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C14">
-        <v>31.18</v>
+        <v>35.33</v>
       </c>
       <c r="D14" t="s">
         <v>24</v>
@@ -1051,13 +1068,13 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C15">
-        <v>36.97</v>
+        <v>31.18</v>
       </c>
       <c r="D15" t="s">
         <v>24</v>
@@ -1068,13 +1085,13 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C16">
-        <v>29.91</v>
+        <v>36.97</v>
       </c>
       <c r="D16" t="s">
         <v>24</v>
@@ -1085,13 +1102,13 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C17">
-        <v>44.48</v>
+        <v>29.91</v>
       </c>
       <c r="D17" t="s">
         <v>24</v>
@@ -1102,13 +1119,13 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C18">
-        <v>36.1</v>
+        <v>44.48</v>
       </c>
       <c r="D18" t="s">
         <v>24</v>
@@ -1119,13 +1136,13 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C19">
-        <v>46.7</v>
+        <v>36.1</v>
       </c>
       <c r="D19" t="s">
         <v>24</v>
@@ -1136,13 +1153,13 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C20">
-        <v>37.619999999999997</v>
+        <v>46.7</v>
       </c>
       <c r="D20" t="s">
         <v>24</v>
@@ -1153,30 +1170,30 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B21" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C21">
-        <v>19.43</v>
+        <v>37.619999999999997</v>
       </c>
       <c r="D21" t="s">
         <v>24</v>
       </c>
       <c r="E21" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B22" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C22">
-        <v>13.44</v>
+        <v>19.43</v>
       </c>
       <c r="D22" t="s">
         <v>24</v>
@@ -1187,13 +1204,13 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B23" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C23">
-        <v>22.69</v>
+        <v>13.44</v>
       </c>
       <c r="D23" t="s">
         <v>24</v>
@@ -1204,13 +1221,13 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B24" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C24">
-        <v>13.62</v>
+        <v>22.69</v>
       </c>
       <c r="D24" t="s">
         <v>24</v>
@@ -1221,13 +1238,13 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B25" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C25">
-        <v>20.22</v>
+        <v>13.62</v>
       </c>
       <c r="D25" t="s">
         <v>24</v>
@@ -1238,13 +1255,13 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B26" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C26">
-        <v>13.48</v>
+        <v>20.22</v>
       </c>
       <c r="D26" t="s">
         <v>24</v>
@@ -1255,13 +1272,13 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B27" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C27">
-        <v>15.22</v>
+        <v>13.48</v>
       </c>
       <c r="D27" t="s">
         <v>24</v>
@@ -1272,13 +1289,13 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C28">
-        <v>15.68</v>
+        <v>15.22</v>
       </c>
       <c r="D28" t="s">
         <v>24</v>
@@ -1289,13 +1306,13 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C29">
-        <v>18.98</v>
+        <v>15.68</v>
       </c>
       <c r="D29" t="s">
         <v>24</v>
@@ -1306,13 +1323,13 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C30">
-        <v>17.149999999999999</v>
+        <v>18.98</v>
       </c>
       <c r="D30" t="s">
         <v>24</v>
@@ -1323,13 +1340,13 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C31">
-        <v>22.04</v>
+        <v>17.149999999999999</v>
       </c>
       <c r="D31" t="s">
         <v>24</v>
@@ -1340,13 +1357,13 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B32" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C32">
-        <v>16.989999999999998</v>
+        <v>22.04</v>
       </c>
       <c r="D32" t="s">
         <v>24</v>
@@ -1357,13 +1374,13 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B33" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C33">
-        <v>24.01</v>
+        <v>16.989999999999998</v>
       </c>
       <c r="D33" t="s">
         <v>24</v>
@@ -1374,13 +1391,13 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C34">
-        <v>18.54</v>
+        <v>24.01</v>
       </c>
       <c r="D34" t="s">
         <v>24</v>
@@ -1391,13 +1408,13 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B35" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C35">
-        <v>31.11</v>
+        <v>18.54</v>
       </c>
       <c r="D35" t="s">
         <v>24</v>
@@ -1408,13 +1425,13 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B36" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C36">
-        <v>32.06</v>
+        <v>31.11</v>
       </c>
       <c r="D36" t="s">
         <v>24</v>
@@ -1425,42 +1442,42 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>68</v>
+      </c>
+      <c r="B37" t="s">
+        <v>19</v>
+      </c>
+      <c r="C37">
+        <v>32.06</v>
+      </c>
+      <c r="D37" t="s">
+        <v>24</v>
+      </c>
+      <c r="E37" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
         <v>30</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B38" t="s">
         <v>3</v>
       </c>
-      <c r="C37">
+      <c r="C38">
         <f>400*24</f>
         <v>9600</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D38" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>67</v>
-      </c>
-      <c r="B38" t="s">
-        <v>4</v>
-      </c>
-      <c r="C38" s="1">
-        <v>2.5</v>
-      </c>
-      <c r="D38" t="s">
-        <v>56</v>
-      </c>
-      <c r="F38" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B39" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C39" s="1">
         <v>2.5</v>
@@ -1474,10 +1491,10 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B40" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C40" s="1">
         <v>2.5</v>
@@ -1491,10 +1508,10 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B41" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C41" s="1">
         <v>2.5</v>
@@ -1508,10 +1525,10 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B42" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C42" s="1">
         <v>2.5</v>
@@ -1525,10 +1542,10 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B43" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C43" s="1">
         <v>2.5</v>
@@ -1542,10 +1559,10 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B44" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C44" s="1">
         <v>2.5</v>
@@ -1559,10 +1576,10 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B45" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C45" s="1">
         <v>2.5</v>
@@ -1576,10 +1593,10 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B46" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C46" s="1">
         <v>2.5</v>
@@ -1593,13 +1610,13 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B47" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C47" s="1">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="D47" t="s">
         <v>56</v>
@@ -1610,10 +1627,10 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B48" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C48" s="1">
         <v>3</v>
@@ -1627,10 +1644,10 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C49" s="1">
         <v>3</v>
@@ -1644,10 +1661,10 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B50" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C50" s="1">
         <v>3</v>
@@ -1661,10 +1678,10 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B51" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C51" s="1">
         <v>3</v>
@@ -1678,10 +1695,10 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B52" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C52" s="1">
         <v>3</v>
@@ -1695,10 +1712,10 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B53" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C53" s="1">
         <v>3</v>
@@ -1708,6 +1725,34 @@
       </c>
       <c r="F53" t="s">
         <v>54</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>68</v>
+      </c>
+      <c r="B54" t="s">
+        <v>19</v>
+      </c>
+      <c r="C54" s="1">
+        <v>3</v>
+      </c>
+      <c r="D54" t="s">
+        <v>56</v>
+      </c>
+      <c r="F54" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>65</v>
+      </c>
+      <c r="C55" s="1">
+        <v>1</v>
+      </c>
+      <c r="F55" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1718,7 +1763,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D254DEF8-D70B-44A9-90B7-19C720405132}">
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F115"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
@@ -2372,7 +2417,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B50" t="s">
         <v>4</v>
@@ -2389,7 +2434,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B51" t="s">
         <v>5</v>
@@ -2406,7 +2451,7 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B52" t="s">
         <v>6</v>
@@ -2423,7 +2468,7 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B53" t="s">
         <v>7</v>
@@ -2440,7 +2485,7 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B54" t="s">
         <v>8</v>
@@ -2457,7 +2502,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B55" t="s">
         <v>9</v>
@@ -2474,7 +2519,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B56" t="s">
         <v>10</v>
@@ -2491,7 +2536,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B57" t="s">
         <v>11</v>
@@ -2508,7 +2553,7 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B58" t="s">
         <v>12</v>
@@ -2525,7 +2570,7 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B59" t="s">
         <v>13</v>
@@ -2542,7 +2587,7 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B60" t="s">
         <v>14</v>
@@ -2559,7 +2604,7 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B61" t="s">
         <v>15</v>
@@ -2576,7 +2621,7 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B62" t="s">
         <v>16</v>
@@ -2593,7 +2638,7 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B63" t="s">
         <v>17</v>
@@ -2610,7 +2655,7 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B64" t="s">
         <v>18</v>
@@ -2627,7 +2672,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B65" t="s">
         <v>19</v>
@@ -2644,7 +2689,7 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B66" t="s">
         <v>4</v>
@@ -2661,7 +2706,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B67" t="s">
         <v>5</v>
@@ -2678,7 +2723,7 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B68" t="s">
         <v>6</v>
@@ -2695,7 +2740,7 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B69" t="s">
         <v>7</v>
@@ -2712,7 +2757,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B70" t="s">
         <v>8</v>
@@ -2729,7 +2774,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B71" t="s">
         <v>9</v>
@@ -2746,7 +2791,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B72" t="s">
         <v>10</v>
@@ -2763,7 +2808,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B73" t="s">
         <v>11</v>
@@ -2780,7 +2825,7 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B74" t="s">
         <v>12</v>
@@ -2797,7 +2842,7 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B75" t="s">
         <v>13</v>
@@ -2814,7 +2859,7 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B76" t="s">
         <v>14</v>
@@ -2831,7 +2876,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B77" t="s">
         <v>15</v>
@@ -2848,7 +2893,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B78" t="s">
         <v>16</v>
@@ -2865,7 +2910,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B79" t="s">
         <v>17</v>
@@ -2882,7 +2927,7 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B80" t="s">
         <v>18</v>
@@ -2899,7 +2944,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B81" t="s">
         <v>19</v>
@@ -2945,7 +2990,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B84" t="s">
         <v>4</v>
@@ -2962,7 +3007,7 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B85" t="s">
         <v>5</v>
@@ -2979,7 +3024,7 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B86" t="s">
         <v>6</v>
@@ -2996,7 +3041,7 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B87" t="s">
         <v>7</v>
@@ -3013,7 +3058,7 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B88" t="s">
         <v>8</v>
@@ -3030,7 +3075,7 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B89" t="s">
         <v>9</v>
@@ -3047,7 +3092,7 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B90" t="s">
         <v>10</v>
@@ -3064,7 +3109,7 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B91" t="s">
         <v>11</v>
@@ -3081,7 +3126,7 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B92" t="s">
         <v>12</v>
@@ -3098,7 +3143,7 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B93" t="s">
         <v>13</v>
@@ -3115,7 +3160,7 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B94" t="s">
         <v>14</v>
@@ -3132,7 +3177,7 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B95" t="s">
         <v>15</v>
@@ -3149,7 +3194,7 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B96" t="s">
         <v>16</v>
@@ -3166,7 +3211,7 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B97" t="s">
         <v>17</v>
@@ -3183,7 +3228,7 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B98" t="s">
         <v>18</v>
@@ -3200,7 +3245,7 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B99" t="s">
         <v>19</v>
@@ -3213,6 +3258,278 @@
       </c>
       <c r="F99" t="s">
         <v>54</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>20</v>
+      </c>
+      <c r="B100" t="s">
+        <v>4</v>
+      </c>
+      <c r="C100">
+        <v>2000</v>
+      </c>
+      <c r="D100" t="s">
+        <v>81</v>
+      </c>
+      <c r="F100" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>20</v>
+      </c>
+      <c r="B101" t="s">
+        <v>5</v>
+      </c>
+      <c r="C101">
+        <v>2000</v>
+      </c>
+      <c r="D101" t="s">
+        <v>81</v>
+      </c>
+      <c r="F101" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>20</v>
+      </c>
+      <c r="B102" t="s">
+        <v>6</v>
+      </c>
+      <c r="C102">
+        <v>2000</v>
+      </c>
+      <c r="D102" t="s">
+        <v>81</v>
+      </c>
+      <c r="F102" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>20</v>
+      </c>
+      <c r="B103" t="s">
+        <v>7</v>
+      </c>
+      <c r="C103">
+        <v>2000</v>
+      </c>
+      <c r="D103" t="s">
+        <v>81</v>
+      </c>
+      <c r="F103" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>20</v>
+      </c>
+      <c r="B104" t="s">
+        <v>8</v>
+      </c>
+      <c r="C104">
+        <v>2000</v>
+      </c>
+      <c r="D104" t="s">
+        <v>81</v>
+      </c>
+      <c r="F104" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>20</v>
+      </c>
+      <c r="B105" t="s">
+        <v>9</v>
+      </c>
+      <c r="C105">
+        <v>2000</v>
+      </c>
+      <c r="D105" t="s">
+        <v>81</v>
+      </c>
+      <c r="F105" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
+        <v>20</v>
+      </c>
+      <c r="B106" t="s">
+        <v>10</v>
+      </c>
+      <c r="C106">
+        <v>2000</v>
+      </c>
+      <c r="D106" t="s">
+        <v>81</v>
+      </c>
+      <c r="F106" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>20</v>
+      </c>
+      <c r="B107" t="s">
+        <v>11</v>
+      </c>
+      <c r="C107">
+        <v>2000</v>
+      </c>
+      <c r="D107" t="s">
+        <v>81</v>
+      </c>
+      <c r="F107" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>20</v>
+      </c>
+      <c r="B108" t="s">
+        <v>12</v>
+      </c>
+      <c r="C108">
+        <v>2000</v>
+      </c>
+      <c r="D108" t="s">
+        <v>81</v>
+      </c>
+      <c r="F108" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>20</v>
+      </c>
+      <c r="B109" t="s">
+        <v>13</v>
+      </c>
+      <c r="C109">
+        <v>2000</v>
+      </c>
+      <c r="D109" t="s">
+        <v>81</v>
+      </c>
+      <c r="F109" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
+        <v>20</v>
+      </c>
+      <c r="B110" t="s">
+        <v>14</v>
+      </c>
+      <c r="C110">
+        <v>2000</v>
+      </c>
+      <c r="D110" t="s">
+        <v>81</v>
+      </c>
+      <c r="F110" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>20</v>
+      </c>
+      <c r="B111" t="s">
+        <v>15</v>
+      </c>
+      <c r="C111">
+        <v>2000</v>
+      </c>
+      <c r="D111" t="s">
+        <v>81</v>
+      </c>
+      <c r="F111" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>20</v>
+      </c>
+      <c r="B112" t="s">
+        <v>16</v>
+      </c>
+      <c r="C112">
+        <v>2000</v>
+      </c>
+      <c r="D112" t="s">
+        <v>81</v>
+      </c>
+      <c r="F112" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>20</v>
+      </c>
+      <c r="B113" t="s">
+        <v>17</v>
+      </c>
+      <c r="C113">
+        <v>2000</v>
+      </c>
+      <c r="D113" t="s">
+        <v>81</v>
+      </c>
+      <c r="F113" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>20</v>
+      </c>
+      <c r="B114" t="s">
+        <v>18</v>
+      </c>
+      <c r="C114">
+        <v>2000</v>
+      </c>
+      <c r="D114" t="s">
+        <v>81</v>
+      </c>
+      <c r="F114" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
+        <v>20</v>
+      </c>
+      <c r="B115" t="s">
+        <v>19</v>
+      </c>
+      <c r="C115">
+        <v>2000</v>
+      </c>
+      <c r="D115" t="s">
+        <v>81</v>
+      </c>
+      <c r="F115" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -3281,7 +3598,7 @@
       </c>
       <c r="G2" s="2"/>
       <c r="I2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -3300,7 +3617,7 @@
       </c>
       <c r="G3" s="2"/>
       <c r="I3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -3319,7 +3636,7 @@
       </c>
       <c r="G4" s="2"/>
       <c r="I4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -3338,7 +3655,7 @@
       </c>
       <c r="G5" s="2"/>
       <c r="I5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -3357,7 +3674,7 @@
       </c>
       <c r="G6" s="2"/>
       <c r="I6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -3376,7 +3693,7 @@
       </c>
       <c r="G7" s="2"/>
       <c r="I7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -3395,7 +3712,7 @@
       </c>
       <c r="G8" s="2"/>
       <c r="I8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -3414,7 +3731,7 @@
       </c>
       <c r="G9" s="2"/>
       <c r="I9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -3433,7 +3750,7 @@
       </c>
       <c r="G10" s="2"/>
       <c r="I10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -3452,7 +3769,7 @@
       </c>
       <c r="G11" s="2"/>
       <c r="I11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -3471,7 +3788,7 @@
       </c>
       <c r="G12" s="2"/>
       <c r="I12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -3490,7 +3807,7 @@
       </c>
       <c r="G13" s="2"/>
       <c r="I13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -3509,7 +3826,7 @@
       </c>
       <c r="G14" s="2"/>
       <c r="I14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
@@ -3528,7 +3845,7 @@
       </c>
       <c r="G15" s="2"/>
       <c r="I15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
@@ -3547,7 +3864,7 @@
       </c>
       <c r="G16" s="2"/>
       <c r="I16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
@@ -3566,7 +3883,7 @@
       </c>
       <c r="G17" s="2"/>
       <c r="I17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
@@ -3585,7 +3902,7 @@
       </c>
       <c r="G18" s="2"/>
       <c r="I18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
@@ -3604,7 +3921,7 @@
       </c>
       <c r="G19" s="2"/>
       <c r="I19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
@@ -3623,7 +3940,7 @@
       </c>
       <c r="G20" s="2"/>
       <c r="I20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
@@ -3642,7 +3959,7 @@
       </c>
       <c r="G21" s="2"/>
       <c r="I21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
@@ -3661,7 +3978,7 @@
       </c>
       <c r="G22" s="2"/>
       <c r="I22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
@@ -3680,7 +3997,7 @@
       </c>
       <c r="G23" s="2"/>
       <c r="I23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
@@ -3699,7 +4016,7 @@
       </c>
       <c r="G24" s="2"/>
       <c r="I24" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
@@ -3718,7 +4035,7 @@
       </c>
       <c r="G25" s="2"/>
       <c r="I25" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
@@ -3737,7 +4054,7 @@
       </c>
       <c r="G26" s="2"/>
       <c r="I26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
@@ -3756,7 +4073,7 @@
       </c>
       <c r="G27" s="2"/>
       <c r="I27" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
@@ -3778,13 +4095,13 @@
         <v>34</v>
       </c>
       <c r="C29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F29">
         <v>10</v>
       </c>
       <c r="I29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
@@ -3792,13 +4109,13 @@
         <v>35</v>
       </c>
       <c r="C30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F30">
         <v>10</v>
       </c>
       <c r="I30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
@@ -3806,13 +4123,13 @@
         <v>36</v>
       </c>
       <c r="C31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F31">
         <v>10</v>
       </c>
       <c r="I31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
@@ -3820,13 +4137,13 @@
         <v>37</v>
       </c>
       <c r="C32" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F32">
         <v>10</v>
       </c>
       <c r="I32" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
@@ -3834,13 +4151,13 @@
         <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F33">
         <v>10</v>
       </c>
       <c r="I33" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
@@ -3848,13 +4165,13 @@
         <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F34">
         <v>10</v>
       </c>
       <c r="I34" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
@@ -3862,13 +4179,13 @@
         <v>57</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F35">
         <v>10</v>
       </c>
       <c r="I35" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
@@ -3876,13 +4193,13 @@
         <v>58</v>
       </c>
       <c r="C36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F36">
         <v>10</v>
       </c>
       <c r="I36" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
@@ -3890,13 +4207,13 @@
         <v>40</v>
       </c>
       <c r="C37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F37">
         <v>10</v>
       </c>
       <c r="I37" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
@@ -3904,13 +4221,13 @@
         <v>41</v>
       </c>
       <c r="C38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F38">
         <v>10</v>
       </c>
       <c r="I38" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
@@ -3918,13 +4235,13 @@
         <v>59</v>
       </c>
       <c r="C39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F39">
         <v>10</v>
       </c>
       <c r="I39" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
@@ -3932,13 +4249,13 @@
         <v>42</v>
       </c>
       <c r="C40" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F40">
         <v>10</v>
       </c>
       <c r="I40" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
@@ -3946,13 +4263,13 @@
         <v>43</v>
       </c>
       <c r="C41" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F41">
         <v>10</v>
       </c>
       <c r="I41" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
@@ -3960,13 +4277,13 @@
         <v>44</v>
       </c>
       <c r="C42" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F42">
         <v>10</v>
       </c>
       <c r="I42" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
@@ -3974,13 +4291,13 @@
         <v>45</v>
       </c>
       <c r="C43" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F43">
         <v>10</v>
       </c>
       <c r="I43" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
@@ -3988,13 +4305,13 @@
         <v>46</v>
       </c>
       <c r="C44" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F44">
         <v>10</v>
       </c>
       <c r="I44" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
@@ -4002,13 +4319,13 @@
         <v>47</v>
       </c>
       <c r="C45" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F45">
         <v>10</v>
       </c>
       <c r="I45" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
@@ -4016,13 +4333,13 @@
         <v>60</v>
       </c>
       <c r="C46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F46">
         <v>10</v>
       </c>
       <c r="I46" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
@@ -4030,13 +4347,13 @@
         <v>48</v>
       </c>
       <c r="C47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F47">
         <v>10</v>
       </c>
       <c r="I47" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
@@ -4044,13 +4361,13 @@
         <v>49</v>
       </c>
       <c r="C48" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F48">
         <v>10</v>
       </c>
       <c r="I48" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
@@ -4058,13 +4375,13 @@
         <v>50</v>
       </c>
       <c r="C49" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F49">
         <v>10</v>
       </c>
       <c r="I49" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
@@ -4072,13 +4389,13 @@
         <v>51</v>
       </c>
       <c r="C50" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F50">
         <v>10</v>
       </c>
       <c r="I50" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
@@ -4086,13 +4403,13 @@
         <v>52</v>
       </c>
       <c r="C51" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F51">
         <v>10</v>
       </c>
       <c r="I51" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
@@ -4100,13 +4417,13 @@
         <v>53</v>
       </c>
       <c r="C52" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F52">
         <v>10</v>
       </c>
       <c r="I52" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
@@ -4114,13 +4431,13 @@
         <v>61</v>
       </c>
       <c r="C53" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F53">
         <v>10</v>
       </c>
       <c r="I53" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
@@ -4128,13 +4445,13 @@
         <v>62</v>
       </c>
       <c r="C54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F54">
         <v>10</v>
       </c>
       <c r="I54" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
@@ -4142,13 +4459,13 @@
         <v>34</v>
       </c>
       <c r="C55" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F55">
         <v>60</v>
       </c>
       <c r="I55" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
@@ -4156,7 +4473,7 @@
         <v>35</v>
       </c>
       <c r="C56" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F56">
         <v>60</v>
@@ -4167,7 +4484,7 @@
         <v>36</v>
       </c>
       <c r="C57" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F57">
         <v>60</v>
@@ -4178,7 +4495,7 @@
         <v>37</v>
       </c>
       <c r="C58" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F58">
         <v>60</v>
@@ -4189,7 +4506,7 @@
         <v>38</v>
       </c>
       <c r="C59" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F59">
         <v>60</v>
@@ -4200,7 +4517,7 @@
         <v>39</v>
       </c>
       <c r="C60" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F60">
         <v>60</v>
@@ -4211,7 +4528,7 @@
         <v>57</v>
       </c>
       <c r="C61" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F61">
         <v>60</v>
@@ -4222,7 +4539,7 @@
         <v>58</v>
       </c>
       <c r="C62" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F62">
         <v>60</v>
@@ -4233,7 +4550,7 @@
         <v>40</v>
       </c>
       <c r="C63" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F63">
         <v>60</v>
@@ -4244,7 +4561,7 @@
         <v>41</v>
       </c>
       <c r="C64" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F64">
         <v>60</v>
@@ -4255,7 +4572,7 @@
         <v>59</v>
       </c>
       <c r="C65" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F65">
         <v>60</v>
@@ -4266,7 +4583,7 @@
         <v>42</v>
       </c>
       <c r="C66" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F66">
         <v>60</v>
@@ -4277,7 +4594,7 @@
         <v>43</v>
       </c>
       <c r="C67" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F67">
         <v>60</v>
@@ -4288,7 +4605,7 @@
         <v>44</v>
       </c>
       <c r="C68" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F68">
         <v>60</v>
@@ -4299,7 +4616,7 @@
         <v>45</v>
       </c>
       <c r="C69" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F69">
         <v>60</v>
@@ -4310,7 +4627,7 @@
         <v>46</v>
       </c>
       <c r="C70" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F70">
         <v>60</v>
@@ -4321,7 +4638,7 @@
         <v>47</v>
       </c>
       <c r="C71" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F71">
         <v>60</v>
@@ -4332,7 +4649,7 @@
         <v>60</v>
       </c>
       <c r="C72" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F72">
         <v>60</v>
@@ -4343,7 +4660,7 @@
         <v>48</v>
       </c>
       <c r="C73" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F73">
         <v>60</v>
@@ -4354,7 +4671,7 @@
         <v>49</v>
       </c>
       <c r="C74" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F74">
         <v>60</v>
@@ -4365,7 +4682,7 @@
         <v>50</v>
       </c>
       <c r="C75" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F75">
         <v>60</v>
@@ -4376,7 +4693,7 @@
         <v>51</v>
       </c>
       <c r="C76" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F76">
         <v>60</v>
@@ -4387,7 +4704,7 @@
         <v>52</v>
       </c>
       <c r="C77" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F77">
         <v>60</v>
@@ -4398,7 +4715,7 @@
         <v>53</v>
       </c>
       <c r="C78" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F78">
         <v>60</v>
@@ -4409,7 +4726,7 @@
         <v>61</v>
       </c>
       <c r="C79" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F79">
         <v>60</v>
@@ -4420,7 +4737,7 @@
         <v>62</v>
       </c>
       <c r="C80" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F80">
         <v>60</v>
@@ -4431,13 +4748,13 @@
         <v>58</v>
       </c>
       <c r="C81" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F81">
         <v>12</v>
       </c>
       <c r="I81" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.3">
@@ -4445,13 +4762,13 @@
         <v>58</v>
       </c>
       <c r="C82" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F82">
         <v>12</v>
       </c>
       <c r="I82" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.3">
@@ -4462,13 +4779,13 @@
         <v>4</v>
       </c>
       <c r="C83" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F83">
         <v>10</v>
       </c>
       <c r="I83" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.3">
@@ -4479,13 +4796,13 @@
         <v>5</v>
       </c>
       <c r="C84" t="s">
+        <v>74</v>
+      </c>
+      <c r="F84">
+        <v>20</v>
+      </c>
+      <c r="I84" t="s">
         <v>75</v>
-      </c>
-      <c r="F84">
-        <v>20</v>
-      </c>
-      <c r="I84" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.3">
@@ -4496,13 +4813,13 @@
         <v>6</v>
       </c>
       <c r="C85" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F85">
         <v>30</v>
       </c>
       <c r="I85" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.3">
@@ -4510,10 +4827,10 @@
         <v>34</v>
       </c>
       <c r="C86" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I86" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.3">
@@ -4521,10 +4838,10 @@
         <v>35</v>
       </c>
       <c r="C87" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I87" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.3">
@@ -4532,10 +4849,10 @@
         <v>36</v>
       </c>
       <c r="C88" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I88" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -4562,7 +4879,7 @@
         <v>63</v>
       </c>
       <c r="C1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D1" t="s">
         <v>55</v>
@@ -4580,7 +4897,7 @@
         <v>68006.708824511996</v>
       </c>
       <c r="D2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
SFm.py: Normunit logic update, CEDARS data field name update
For SFM.py, this update includes:
1. normalizing unit lookup logic / validation update
2. CEDARS data field name update "Type (Whole Building or End Use)"
</commit_message>
<xml_diff>
--- a/scripts/data transformation/Normunits.xlsx
+++ b/scripts/data transformation/Normunits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YLIAN\Documents\DEER_github_apr26\DEER-Prototypes-EnergyPlus\scripts\data transformation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FE080E6-8019-465C-8D28-A823225A6BBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B72654-5320-466A-B69E-8B0B918500A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{527A75FC-5BC9-4372-9120-09678A46B600}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{527A75FC-5BC9-4372-9120-09678A46B600}"/>
   </bookViews>
   <sheets>
     <sheet name="DMo" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="Com_area" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">SFm!$A$1:$F$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">SFm!$A$1:$F$100</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="83">
   <si>
     <t>Normunit</t>
   </si>
@@ -1763,7 +1763,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D254DEF8-D70B-44A9-90B7-19C720405132}">
-  <dimension ref="A1:F115"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
@@ -2990,19 +2990,13 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B84" t="s">
-        <v>4</v>
-      </c>
-      <c r="C84" s="1">
-        <v>4</v>
-      </c>
-      <c r="D84" t="s">
-        <v>56</v>
-      </c>
-      <c r="F84" t="s">
-        <v>54</v>
+        <v>3</v>
+      </c>
+      <c r="C84">
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
@@ -3010,7 +3004,7 @@
         <v>68</v>
       </c>
       <c r="B85" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C85" s="1">
         <v>4</v>
@@ -3027,7 +3021,7 @@
         <v>68</v>
       </c>
       <c r="B86" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C86" s="1">
         <v>4</v>
@@ -3044,7 +3038,7 @@
         <v>68</v>
       </c>
       <c r="B87" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C87" s="1">
         <v>4</v>
@@ -3061,7 +3055,7 @@
         <v>68</v>
       </c>
       <c r="B88" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C88" s="1">
         <v>4</v>
@@ -3078,7 +3072,7 @@
         <v>68</v>
       </c>
       <c r="B89" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C89" s="1">
         <v>4</v>
@@ -3095,7 +3089,7 @@
         <v>68</v>
       </c>
       <c r="B90" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C90" s="1">
         <v>4</v>
@@ -3112,7 +3106,7 @@
         <v>68</v>
       </c>
       <c r="B91" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C91" s="1">
         <v>4</v>
@@ -3129,7 +3123,7 @@
         <v>68</v>
       </c>
       <c r="B92" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C92" s="1">
         <v>4</v>
@@ -3146,10 +3140,10 @@
         <v>68</v>
       </c>
       <c r="B93" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C93" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D93" t="s">
         <v>56</v>
@@ -3163,7 +3157,7 @@
         <v>68</v>
       </c>
       <c r="B94" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C94" s="1">
         <v>5</v>
@@ -3180,7 +3174,7 @@
         <v>68</v>
       </c>
       <c r="B95" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C95" s="1">
         <v>5</v>
@@ -3197,7 +3191,7 @@
         <v>68</v>
       </c>
       <c r="B96" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C96" s="1">
         <v>5</v>
@@ -3214,7 +3208,7 @@
         <v>68</v>
       </c>
       <c r="B97" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C97" s="1">
         <v>5</v>
@@ -3231,7 +3225,7 @@
         <v>68</v>
       </c>
       <c r="B98" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C98" s="1">
         <v>5</v>
@@ -3248,7 +3242,7 @@
         <v>68</v>
       </c>
       <c r="B99" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C99" s="1">
         <v>5</v>
@@ -3262,19 +3256,19 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="B100" t="s">
-        <v>4</v>
-      </c>
-      <c r="C100">
-        <v>2000</v>
+        <v>19</v>
+      </c>
+      <c r="C100" s="1">
+        <v>5</v>
       </c>
       <c r="D100" t="s">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="F100" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
@@ -3282,7 +3276,7 @@
         <v>20</v>
       </c>
       <c r="B101" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C101">
         <v>2000</v>
@@ -3299,7 +3293,7 @@
         <v>20</v>
       </c>
       <c r="B102" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C102">
         <v>2000</v>
@@ -3316,7 +3310,7 @@
         <v>20</v>
       </c>
       <c r="B103" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C103">
         <v>2000</v>
@@ -3333,7 +3327,7 @@
         <v>20</v>
       </c>
       <c r="B104" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C104">
         <v>2000</v>
@@ -3350,7 +3344,7 @@
         <v>20</v>
       </c>
       <c r="B105" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C105">
         <v>2000</v>
@@ -3367,7 +3361,7 @@
         <v>20</v>
       </c>
       <c r="B106" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C106">
         <v>2000</v>
@@ -3384,7 +3378,7 @@
         <v>20</v>
       </c>
       <c r="B107" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C107">
         <v>2000</v>
@@ -3401,7 +3395,7 @@
         <v>20</v>
       </c>
       <c r="B108" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C108">
         <v>2000</v>
@@ -3418,7 +3412,7 @@
         <v>20</v>
       </c>
       <c r="B109" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C109">
         <v>2000</v>
@@ -3435,7 +3429,7 @@
         <v>20</v>
       </c>
       <c r="B110" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C110">
         <v>2000</v>
@@ -3452,7 +3446,7 @@
         <v>20</v>
       </c>
       <c r="B111" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C111">
         <v>2000</v>
@@ -3469,7 +3463,7 @@
         <v>20</v>
       </c>
       <c r="B112" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C112">
         <v>2000</v>
@@ -3486,7 +3480,7 @@
         <v>20</v>
       </c>
       <c r="B113" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C113">
         <v>2000</v>
@@ -3503,7 +3497,7 @@
         <v>20</v>
       </c>
       <c r="B114" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C114">
         <v>2000</v>
@@ -3520,7 +3514,7 @@
         <v>20</v>
       </c>
       <c r="B115" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C115">
         <v>2000</v>
@@ -3532,8 +3526,25 @@
         <v>82</v>
       </c>
     </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
+        <v>20</v>
+      </c>
+      <c r="B116" t="s">
+        <v>19</v>
+      </c>
+      <c r="C116">
+        <v>2000</v>
+      </c>
+      <c r="D116" t="s">
+        <v>81</v>
+      </c>
+      <c r="F116" t="s">
+        <v>82</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F99" xr:uid="{D254DEF8-D70B-44A9-90B7-19C720405132}"/>
+  <autoFilter ref="A1:F100" xr:uid="{D254DEF8-D70B-44A9-90B7-19C720405132}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
DMo.py: Normunit logic update, CEDARS data field name update
For DMo.py, this update includes:
1. normalizing unit lookup logic / validation update
2. CEDARS data field name update "Type (Whole Building or End Use)"
</commit_message>
<xml_diff>
--- a/scripts/data transformation/Normunits.xlsx
+++ b/scripts/data transformation/Normunits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YLIAN\Documents\DEER_github_apr26\DEER-Prototypes-EnergyPlus\scripts\data transformation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B72654-5320-466A-B69E-8B0B918500A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F97F49B3-EC2C-4E4A-B881-009059119872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{527A75FC-5BC9-4372-9120-09678A46B600}"/>
+    <workbookView xWindow="3372" yWindow="1320" windowWidth="17280" windowHeight="8988" xr2:uid="{527A75FC-5BC9-4372-9120-09678A46B600}"/>
   </bookViews>
   <sheets>
     <sheet name="DMo" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="83">
   <si>
     <t>Normunit</t>
   </si>
@@ -710,14 +710,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2593147D-FBCE-4A43-B94C-18CB04EC4F0B}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -725,101 +725,115 @@
         <v>32</v>
       </c>
       <c r="C1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>21</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>2480</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>20</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>2174.56</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>20</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>2480</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>20</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>2000</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>81</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>30</v>
       </c>
       <c r="B6" t="s">
         <v>3</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <f>400*2</f>
         <v>800</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>68</v>
       </c>
       <c r="B7" t="s">
         <v>3</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>3.5</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>56</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>